<commit_message>
WIP: import y build historico de tarifas sin terminar
</commit_message>
<xml_diff>
--- a/exports/historical-tariffs-analysis.xlsx
+++ b/exports/historical-tariffs-analysis.xlsx
@@ -606,7 +606,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B5" t="str">
         <v>Bachata en Pareja</v>
@@ -614,11 +614,20 @@
       <c r="C5" t="str">
         <v>MAX</v>
       </c>
+      <c r="D5" t="str">
+        <v>Bachata en Pareja</v>
+      </c>
+      <c r="E5" t="str">
+        <v>d06eb88b-a6e3-4cda-8bf9-5278455b3b7e</v>
+      </c>
+      <c r="F5" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G5" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H5" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I5" t="str">
         <v>2026-02-01</v>
@@ -641,15 +650,6 @@
       <c r="O5" t="str">
         <v>120</v>
       </c>
-      <c r="P5" t="str">
-        <v>Mambo en parejas</v>
-      </c>
-      <c r="Q5" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="R5" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -700,7 +700,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B7" t="str">
         <v>Bachata Pasos Sueltos</v>
@@ -708,11 +708,20 @@
       <c r="C7" t="str">
         <v>MAX</v>
       </c>
+      <c r="D7" t="str">
+        <v>Bachata Pasos Sueltos</v>
+      </c>
+      <c r="E7" t="str">
+        <v>8da07d2d-b252-4618-9370-34f8ca23e93e</v>
+      </c>
+      <c r="F7" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G7" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H7" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I7" t="str">
         <v>2026-02-01</v>
@@ -735,12 +744,6 @@
       <c r="O7" t="str">
         <v>119</v>
       </c>
-      <c r="P7" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="Q7" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -932,7 +935,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B12" t="str">
         <v>Bachata y Salsa Inicial</v>
@@ -979,7 +982,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>OK</v>
       </c>
       <c r="B13" t="str">
         <v>Bachata y Salsa Inicial</v>
@@ -1026,7 +1029,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B14" t="str">
         <v>Belly Dance Alternativo</v>
@@ -1034,11 +1037,20 @@
       <c r="C14" t="str">
         <v>VIRGINIA</v>
       </c>
+      <c r="D14" t="str">
+        <v>Belly Dance Alternativo</v>
+      </c>
+      <c r="E14" t="str">
+        <v>dbd5af21-ec55-4380-8ca1-d643a10d2003</v>
+      </c>
+      <c r="F14" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G14" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H14" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I14" t="str">
         <v>2025-02-01</v>
@@ -1064,7 +1076,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B15" t="str">
         <v>Coreográfico Bachata en Pareja</v>
@@ -1072,11 +1084,20 @@
       <c r="C15" t="str">
         <v>KEVIN</v>
       </c>
+      <c r="D15" t="str">
+        <v>Coreográfico Bachata en Pareja</v>
+      </c>
+      <c r="E15" t="str">
+        <v>28f1b214-f935-4bea-8a8c-a28789592bb0</v>
+      </c>
+      <c r="F15" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G15" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H15" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I15" t="str">
         <v>2025-05-01</v>
@@ -1099,19 +1120,10 @@
       <c r="O15" t="str">
         <v>51</v>
       </c>
-      <c r="P15" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="Q15" t="str">
-        <v>Mambo en parejas</v>
-      </c>
-      <c r="R15" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B16" t="str">
         <v>Coreográfico Bachata en Pareja</v>
@@ -1119,11 +1131,20 @@
       <c r="C16" t="str">
         <v>KEVIN</v>
       </c>
+      <c r="D16" t="str">
+        <v>Coreográfico Bachata en Pareja</v>
+      </c>
+      <c r="E16" t="str">
+        <v>28f1b214-f935-4bea-8a8c-a28789592bb0</v>
+      </c>
+      <c r="F16" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G16" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H16" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I16" t="str">
         <v>2025-06-01</v>
@@ -1146,19 +1167,10 @@
       <c r="O16" t="str">
         <v>64</v>
       </c>
-      <c r="P16" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="Q16" t="str">
-        <v>Mambo en parejas</v>
-      </c>
-      <c r="R16" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>REVIEW_CLASS_AND_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B17" t="str">
         <v>Coreográfico Bachata en Pareja</v>
@@ -1166,11 +1178,20 @@
       <c r="C17" t="str">
         <v>KEVIN</v>
       </c>
+      <c r="D17" t="str">
+        <v>Coreográfico Bachata en Pareja</v>
+      </c>
+      <c r="E17" t="str">
+        <v>28f1b214-f935-4bea-8a8c-a28789592bb0</v>
+      </c>
+      <c r="F17" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G17" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H17" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I17" t="str">
         <v>2025-07-01</v>
@@ -1193,15 +1214,6 @@
       <c r="O17" t="str">
         <v>77</v>
       </c>
-      <c r="P17" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="Q17" t="str">
-        <v>Mambo en parejas</v>
-      </c>
-      <c r="R17" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1440,7 +1452,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B23" t="str">
         <v>Coreográfico Femenino</v>
@@ -1863,7 +1875,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B32" t="str">
         <v>Estilo Femenino</v>
@@ -2051,7 +2063,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B36" t="str">
         <v>Fitdance + Axé</v>
@@ -2059,11 +2071,20 @@
       <c r="C36" t="str">
         <v>JOSELO</v>
       </c>
+      <c r="D36" t="str">
+        <v>Fitdance + Axé</v>
+      </c>
+      <c r="E36" t="str">
+        <v>db1e0e5e-c5e0-429e-aec3-4f28d406dad9</v>
+      </c>
+      <c r="F36" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G36" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H36" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I36" t="str">
         <v>2025-02-01</v>
@@ -2089,7 +2110,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B37" t="str">
         <v>Infantil</v>
@@ -2097,11 +2118,20 @@
       <c r="C37" t="str">
         <v>SANTY</v>
       </c>
+      <c r="D37" t="str">
+        <v>S.C Infantil (6-11 años)</v>
+      </c>
+      <c r="E37" t="str">
+        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
+      </c>
+      <c r="F37" t="str">
+        <v>ACTIVE</v>
+      </c>
       <c r="G37" t="str">
-        <v>NO_MATCH</v>
+        <v>MANUAL_ACTIVITY_TEACHER</v>
       </c>
       <c r="H37" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I37" t="str">
         <v>2025-02-01</v>
@@ -2124,19 +2154,10 @@
       <c r="O37" t="str">
         <v>7</v>
       </c>
-      <c r="P37" t="str">
-        <v>Árabe infantil</v>
-      </c>
-      <c r="Q37" t="str">
-        <v>Infantil (6 a 7 años)</v>
-      </c>
-      <c r="R37" t="str">
-        <v>S.C Infantil (6-11 años)</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B38" t="str">
         <v>Infantil</v>
@@ -2144,11 +2165,20 @@
       <c r="C38" t="str">
         <v>SANTY</v>
       </c>
+      <c r="D38" t="str">
+        <v>S.C Infantil (6-11 años)</v>
+      </c>
+      <c r="E38" t="str">
+        <v>4b2663bf-5ab4-42e5-865c-2af4da2cf5ff</v>
+      </c>
+      <c r="F38" t="str">
+        <v>ACTIVE</v>
+      </c>
       <c r="G38" t="str">
-        <v>NO_MATCH</v>
+        <v>MANUAL_ACTIVITY_TEACHER</v>
       </c>
       <c r="H38" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I38" t="str">
         <v>2025-03-01</v>
@@ -2171,15 +2201,6 @@
       <c r="O38" t="str">
         <v>23, 38</v>
       </c>
-      <c r="P38" t="str">
-        <v>Árabe infantil</v>
-      </c>
-      <c r="Q38" t="str">
-        <v>Infantil (6 a 7 años)</v>
-      </c>
-      <c r="R38" t="str">
-        <v>S.C Infantil (6-11 años)</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -2418,7 +2439,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B44" t="str">
         <v>Infantil</v>
@@ -2653,7 +2674,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B49" t="str">
         <v>Kids</v>
@@ -2841,7 +2862,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B53" t="str">
         <v>Ladys Tango - Gabriela P.</v>
@@ -2849,11 +2870,20 @@
       <c r="C53" t="str">
         <v>GABI</v>
       </c>
+      <c r="D53" t="str">
+        <v>Ladys Tango - Gabriela P.</v>
+      </c>
+      <c r="E53" t="str">
+        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
+      </c>
+      <c r="F53" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G53" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H53" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I53" t="str">
         <v>2025-02-01</v>
@@ -2876,19 +2906,10 @@
       <c r="O53" t="str">
         <v>10</v>
       </c>
-      <c r="P53" t="str">
-        <v>Ladys Kizz</v>
-      </c>
-      <c r="Q53" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="R53" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B54" t="str">
         <v>Ladys Tango - Gabriela P.</v>
@@ -2896,11 +2917,20 @@
       <c r="C54" t="str">
         <v>GABI</v>
       </c>
+      <c r="D54" t="str">
+        <v>Ladys Tango - Gabriela P.</v>
+      </c>
+      <c r="E54" t="str">
+        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
+      </c>
+      <c r="F54" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G54" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H54" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I54" t="str">
         <v>2025-03-01</v>
@@ -2923,19 +2953,10 @@
       <c r="O54" t="str">
         <v>26, 41</v>
       </c>
-      <c r="P54" t="str">
-        <v>Ladys Kizz</v>
-      </c>
-      <c r="Q54" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="R54" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B55" t="str">
         <v>Ladys Tango - Gabriela P.</v>
@@ -2943,11 +2964,20 @@
       <c r="C55" t="str">
         <v>GABI</v>
       </c>
+      <c r="D55" t="str">
+        <v>Ladys Tango - Gabriela P.</v>
+      </c>
+      <c r="E55" t="str">
+        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
+      </c>
+      <c r="F55" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G55" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H55" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I55" t="str">
         <v>2025-05-01</v>
@@ -2970,19 +3000,10 @@
       <c r="O55" t="str">
         <v>57, 70</v>
       </c>
-      <c r="P55" t="str">
-        <v>Ladys Kizz</v>
-      </c>
-      <c r="Q55" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="R55" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B56" t="str">
         <v>Ladys Tango - Gabriela P.</v>
@@ -2990,11 +3011,20 @@
       <c r="C56" t="str">
         <v>GABI</v>
       </c>
+      <c r="D56" t="str">
+        <v>Ladys Tango - Gabriela P.</v>
+      </c>
+      <c r="E56" t="str">
+        <v>a12f5acf-4754-479a-853c-15926c2dac92</v>
+      </c>
+      <c r="F56" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G56" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H56" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I56" t="str">
         <v>2025-07-01</v>
@@ -3017,15 +3047,6 @@
       <c r="O56" t="str">
         <v>83</v>
       </c>
-      <c r="P56" t="str">
-        <v>Ladys Kizz</v>
-      </c>
-      <c r="Q56" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="R56" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -3452,7 +3473,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B66" t="str">
         <v>Mambo en Pareja</v>
@@ -3640,7 +3661,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B70" t="str">
         <v>Salsa Inicial / Siesta</v>
@@ -4110,7 +4131,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B80" t="str">
         <v>Tango Avanzado/Intermedio</v>
@@ -4204,7 +4225,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>REVIEW_CLASS</v>
+        <v>OK</v>
       </c>
       <c r="B82" t="str">
         <v>Tango Inicial</v>
@@ -4212,11 +4233,20 @@
       <c r="C82" t="str">
         <v>GABI</v>
       </c>
+      <c r="D82" t="str">
+        <v>Tango Inicial</v>
+      </c>
+      <c r="E82" t="str">
+        <v>23888530-c53d-4c40-94ee-982518e5d2f6</v>
+      </c>
+      <c r="F82" t="str">
+        <v>INACTIVE</v>
+      </c>
       <c r="G82" t="str">
-        <v>NO_MATCH</v>
+        <v>EXACT_NAME</v>
       </c>
       <c r="H82" t="str">
-        <v>LOW</v>
+        <v>HIGH</v>
       </c>
       <c r="I82" t="str">
         <v>2026-03-01</v>
@@ -4239,15 +4269,6 @@
       <c r="O82" t="str">
         <v>136</v>
       </c>
-      <c r="P82" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="Q82" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="R82" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -4768,7 +4789,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B94" t="str">
         <v>Teens</v>
@@ -4909,7 +4930,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>REVIEW_PRICE</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B97" t="str">
         <v>Zumba</v>
@@ -4986,7 +5007,7 @@
         <v>2026-08-31</v>
       </c>
       <c r="K98" t="str">
-        <v>35000.00</v>
+        <v>40000.00</v>
       </c>
       <c r="L98">
         <v>1</v>
@@ -5010,834 +5031,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Actividad</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Profesor</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Importe candidato</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Vigencia desde</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Sugerencia 1</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Score 1</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Sugerencia 2</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Score 2</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Sugerencia 3</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Score 3</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Bachata en Pareja</v>
-      </c>
-      <c r="B2" t="str">
-        <v>MAX</v>
-      </c>
-      <c r="C2" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="D2" t="str">
-        <v>2026-02-01</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Mambo en parejas</v>
-      </c>
-      <c r="F2">
-        <v>0.2</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="H2">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="J2">
-        <v>0.14285714285714285</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Bachata Pasos Sueltos</v>
-      </c>
-      <c r="B3" t="str">
-        <v>MAX</v>
-      </c>
-      <c r="C3" t="str">
-        <v>30000.00</v>
-      </c>
-      <c r="D3" t="str">
-        <v>2026-02-01</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="F3">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="H3">
-        <v>0.14285714285714285</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Belly Dance Alternativo</v>
-      </c>
-      <c r="B4" t="str">
-        <v>VIRGINIA</v>
-      </c>
-      <c r="C4" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="D4" t="str">
-        <v>2025-02-01</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="B5" t="str">
-        <v>KEVIN</v>
-      </c>
-      <c r="C5" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="D5" t="str">
-        <v>2025-05-01</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="F5">
-        <v>0.2857142857142857</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Mambo en parejas</v>
-      </c>
-      <c r="H5">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="J5">
-        <v>0.14285714285714285</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="B6" t="str">
-        <v>KEVIN</v>
-      </c>
-      <c r="C6" t="str">
-        <v>10000.00</v>
-      </c>
-      <c r="D6" t="str">
-        <v>2025-06-01</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="F6">
-        <v>0.2857142857142857</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Mambo en parejas</v>
-      </c>
-      <c r="H6">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="J6">
-        <v>0.14285714285714285</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="B7" t="str">
-        <v>KEVIN</v>
-      </c>
-      <c r="C7" t="str">
-        <v>5000.00</v>
-      </c>
-      <c r="D7" t="str">
-        <v>2025-07-01</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Coreografico E.Masc-Bachata/Urban</v>
-      </c>
-      <c r="F7">
-        <v>0.2857142857142857</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Mambo en parejas</v>
-      </c>
-      <c r="H7">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="I7" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="J7">
-        <v>0.14285714285714285</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Fitdance + Axé</v>
-      </c>
-      <c r="B8" t="str">
-        <v>JOSELO</v>
-      </c>
-      <c r="C8" t="str">
-        <v>7500.00</v>
-      </c>
-      <c r="D8" t="str">
-        <v>2025-02-01</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Infantil</v>
-      </c>
-      <c r="B9" t="str">
-        <v>SANTY</v>
-      </c>
-      <c r="C9" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="D9" t="str">
-        <v>2025-02-01</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Árabe infantil</v>
-      </c>
-      <c r="F9">
-        <v>0.5</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Infantil (6 a 7 años)</v>
-      </c>
-      <c r="H9">
-        <v>0.2</v>
-      </c>
-      <c r="I9" t="str">
-        <v>S.C Infantil (6-11 años)</v>
-      </c>
-      <c r="J9">
-        <v>0.16666666666666666</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Infantil</v>
-      </c>
-      <c r="B10" t="str">
-        <v>SANTY</v>
-      </c>
-      <c r="C10" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="D10" t="str">
-        <v>2025-03-01</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Árabe infantil</v>
-      </c>
-      <c r="F10">
-        <v>0.5</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Infantil (6 a 7 años)</v>
-      </c>
-      <c r="H10">
-        <v>0.2</v>
-      </c>
-      <c r="I10" t="str">
-        <v>S.C Infantil (6-11 años)</v>
-      </c>
-      <c r="J10">
-        <v>0.16666666666666666</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Ladys Tango - Gabriela P.</v>
-      </c>
-      <c r="B11" t="str">
-        <v>GABI</v>
-      </c>
-      <c r="C11" t="str">
-        <v>7500.00</v>
-      </c>
-      <c r="D11" t="str">
-        <v>2025-02-01</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Ladys Kizz</v>
-      </c>
-      <c r="F11">
-        <v>0.2</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="H11">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="I11" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
-      <c r="J11">
-        <v>0.1111111111111111</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Ladys Tango - Gabriela P.</v>
-      </c>
-      <c r="B12" t="str">
-        <v>GABI</v>
-      </c>
-      <c r="C12" t="str">
-        <v>10000.00</v>
-      </c>
-      <c r="D12" t="str">
-        <v>2025-03-01</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Ladys Kizz</v>
-      </c>
-      <c r="F12">
-        <v>0.2</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="H12">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="I12" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
-      <c r="J12">
-        <v>0.1111111111111111</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Ladys Tango - Gabriela P.</v>
-      </c>
-      <c r="B13" t="str">
-        <v>GABI</v>
-      </c>
-      <c r="C13" t="str">
-        <v>11000.00</v>
-      </c>
-      <c r="D13" t="str">
-        <v>2025-05-01</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Ladys Kizz</v>
-      </c>
-      <c r="F13">
-        <v>0.2</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="H13">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="I13" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
-      <c r="J13">
-        <v>0.1111111111111111</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Ladys Tango - Gabriela P.</v>
-      </c>
-      <c r="B14" t="str">
-        <v>GABI</v>
-      </c>
-      <c r="C14" t="str">
-        <v>20000.00</v>
-      </c>
-      <c r="D14" t="str">
-        <v>2025-07-01</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Ladys Kizz</v>
-      </c>
-      <c r="F14">
-        <v>0.2</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="H14">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="I14" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
-      <c r="J14">
-        <v>0.1111111111111111</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Tango Inicial</v>
-      </c>
-      <c r="B15" t="str">
-        <v>GABI</v>
-      </c>
-      <c r="C15" t="str">
-        <v>30000.00</v>
-      </c>
-      <c r="D15" t="str">
-        <v>2026-03-01</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="F15">
-        <v>0.25</v>
-      </c>
-      <c r="G15" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="H15">
-        <v>0.2</v>
-      </c>
-      <c r="I15" t="str">
-        <v>Inst.Sup.Coreografico -Tango /18 Meses</v>
-      </c>
-      <c r="J15">
-        <v>0.14285714285714285</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Actividad</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Profesor</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Clase</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Vigencia desde</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Vigencia hasta</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Importe</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Confianza</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Revisión</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Filas origen</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="B2" t="str">
-        <v>JOSELO</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="D2" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="E2" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="F2" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="G2" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H2" t="str">
-        <v>REVISAR_JULIO</v>
-      </c>
-      <c r="I2" t="str">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="B3" t="str">
-        <v>JOSELO</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="D3" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="E3" t="str">
-        <v>2026-08-31</v>
-      </c>
-      <c r="F3" t="str">
-        <v>40000.00</v>
-      </c>
-      <c r="G3" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H3" t="str">
-        <v>REVISAR_PRECIO</v>
-      </c>
-      <c r="I3" t="str">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Coreográfico Bachata en Pareja</v>
-      </c>
-      <c r="B4" t="str">
-        <v>KEVIN</v>
-      </c>
-      <c r="D4" t="str">
-        <v>2025-07-01</v>
-      </c>
-      <c r="E4" t="str">
-        <v>2025-07-31</v>
-      </c>
-      <c r="F4" t="str">
-        <v>5000.00</v>
-      </c>
-      <c r="G4" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H4" t="str">
-        <v>REVISAR_PRECIO</v>
-      </c>
-      <c r="I4" t="str">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Coreográfico Femenino</v>
-      </c>
-      <c r="B5" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D5" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="E5" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="F5" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="G5" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H5" t="str">
-        <v>REVISAR_JULIO</v>
-      </c>
-      <c r="I5" t="str">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Estilo Femenino</v>
-      </c>
-      <c r="B6" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Clase femenino Sofi</v>
-      </c>
-      <c r="D6" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="E6" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="F6" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="G6" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H6" t="str">
-        <v>REVISAR_JULIO</v>
-      </c>
-      <c r="I6" t="str">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Infantil</v>
-      </c>
-      <c r="B7" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Infantil (6 a 7 años)</v>
-      </c>
-      <c r="D7" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="E7" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="F7" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="G7" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H7" t="str">
-        <v>REVISAR_JULIO</v>
-      </c>
-      <c r="I7" t="str">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Kids</v>
-      </c>
-      <c r="B8" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Kids 4-5 años</v>
-      </c>
-      <c r="D8" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="E8" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="F8" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="G8" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H8" t="str">
-        <v>REVISAR_JULIO</v>
-      </c>
-      <c r="I8" t="str">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Mambo en Pareja</v>
-      </c>
-      <c r="B9" t="str">
-        <v>FER</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Mambo en parejas</v>
-      </c>
-      <c r="D9" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="E9" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="F9" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="G9" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H9" t="str">
-        <v>REVISAR_JULIO</v>
-      </c>
-      <c r="I9" t="str">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Salsa Inicial / Siesta</v>
-      </c>
-      <c r="B10" t="str">
-        <v>JAVI</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Bachata y Salsa Inicial</v>
-      </c>
-      <c r="D10" t="str">
-        <v>2025-09-01</v>
-      </c>
-      <c r="E10" t="str">
-        <v>2025-09-30</v>
-      </c>
-      <c r="F10" t="str">
-        <v>7500.00</v>
-      </c>
-      <c r="G10" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H10" t="str">
-        <v>REVISAR_PRECIO</v>
-      </c>
-      <c r="I10" t="str">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Tango Avanzado/Intermedio</v>
-      </c>
-      <c r="B11" t="str">
-        <v>ROBERTO</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Tango (Inter/Avanz)</v>
-      </c>
-      <c r="D11" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="E11" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="F11" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="G11" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H11" t="str">
-        <v>REVISAR_JULIO</v>
-      </c>
-      <c r="I11" t="str">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Teens</v>
-      </c>
-      <c r="B12" t="str">
-        <v>SOFIA</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Teens (8 a 12 años)</v>
-      </c>
-      <c r="D12" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="E12" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="F12" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="G12" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H12" t="str">
-        <v>REVISAR_JULIO</v>
-      </c>
-      <c r="I12" t="str">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Zumba</v>
-      </c>
-      <c r="B13" t="str">
-        <v>JOSELO</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Zumba - Profe Joselo</v>
-      </c>
-      <c r="D13" t="str">
-        <v>2026-07-01</v>
-      </c>
-      <c r="E13" t="str">
-        <v>2026-07-31</v>
-      </c>
-      <c r="F13" t="str">
-        <v>15000.00</v>
-      </c>
-      <c r="G13" t="str">
-        <v>BAJA</v>
-      </c>
-      <c r="H13" t="str">
-        <v>REVISAR_JULIO</v>
-      </c>
-      <c r="I13" t="str">
-        <v>168</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5867,7 +5074,7 @@
         <v>OK</v>
       </c>
       <c r="B3">
-        <v>72</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4">
@@ -5875,7 +5082,7 @@
         <v>Revisar precio</v>
       </c>
       <c r="B4">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -5883,7 +5090,7 @@
         <v>Revisar clase</v>
       </c>
       <c r="B5">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -5891,7 +5098,7 @@
         <v>Revisar clase y precio</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
WIP: version cuasi final de las cuotas historicas
</commit_message>
<xml_diff>
--- a/exports/historical-tariffs-analysis.xlsx
+++ b/exports/historical-tariffs-analysis.xlsx
@@ -1311,7 +1311,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>OK</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B20" t="str">
         <v>Coreográfico Femenino</v>
@@ -1358,7 +1358,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>OK</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B21" t="str">
         <v>Coreográfico Femenino</v>
@@ -1640,7 +1640,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>OK</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B27" t="str">
         <v>Estilo Femenino</v>
@@ -1734,7 +1734,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>OK</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B29" t="str">
         <v>Estilo Femenino</v>
@@ -3708,7 +3708,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>OK</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B71" t="str">
         <v>Salsa Inicial / Siesta</v>
@@ -5074,7 +5074,7 @@
         <v>OK</v>
       </c>
       <c r="B3">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
WIP: cambios en Tariff, creación de tarifas históricas para c/clase, y progreso con la implementación de los monthly charges
</commit_message>
<xml_diff>
--- a/exports/historical-tariffs-analysis.xlsx
+++ b/exports/historical-tariffs-analysis.xlsx
@@ -1244,7 +1244,7 @@
         <v>2025-02-01</v>
       </c>
       <c r="J18" t="str">
-        <v>2025-03-31</v>
+        <v>2025-02-28</v>
       </c>
       <c r="K18" t="str">
         <v>15000.00</v>
@@ -1546,7 +1546,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>OK</v>
+        <v>NOT_A_TARIFF</v>
       </c>
       <c r="B25" t="str">
         <v>Estilo Femenino</v>
@@ -5074,7 +5074,7 @@
         <v>OK</v>
       </c>
       <c r="B3">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4">

</xml_diff>